<commit_message>
Savetts 2026: bracket setup, payments and schedule tweaks
Tournament data captured through the control panel:

- Add Men's 40+ and Men's 50+ knockout brackets (16), and seed the Men's Doubles
  bracket -- 8 of its round-1 matches are filled, using direct entry picks since the
  doubles events have no group stage.
- Mark six entries as paid, and correct one entry from Gareth Bunce (Mother City,
  Men's 40+) to Benjamin van der Ross (Livken, Men's 40+ and 50+).
- Turn on group visibility for the public site.
- Adjust one Day 2 11:30 schedule slot, and update Groups.xlsx and Schedule.xlsx to
  match.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Savets 2026/admin/Groups.xlsx
+++ b/Savets 2026/admin/Groups.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C69FF3E6-BF31-4780-827A-748758DFD531}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0EA9C29-9FC4-4D49-8AE5-11666D6838D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9120" yWindow="2190" windowWidth="15300" windowHeight="7785" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Men's 40+" sheetId="4" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="47">
   <si>
     <t>Group 1 Names</t>
   </si>
@@ -133,12 +133,6 @@
     <t>Frans Erasmus</t>
   </si>
   <si>
-    <t>Gareth Bunce</t>
-  </si>
-  <si>
-    <t>Mother City</t>
-  </si>
-  <si>
     <t>Jerome Davies</t>
   </si>
   <si>
@@ -161,6 +155,9 @@
   </si>
   <si>
     <t>Amien Phillips</t>
+  </si>
+  <si>
+    <t>Benjamin van der Ross</t>
   </si>
 </sst>
 </file>
@@ -339,7 +336,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -684,7 +681,7 @@
   <dimension ref="A1:L17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.5703125" customWidth="1"/>
     <col min="2" max="2" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -826,28 +823,28 @@
         <v>30</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>30</v>
       </c>
       <c r="G4" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I4" s="9" t="s">
         <v>40</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="I4" s="9" t="s">
-        <v>42</v>
       </c>
       <c r="J4" s="5" t="s">
         <v>17</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -858,13 +855,13 @@
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
       <c r="I5" s="9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="J5" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="K5" s="12" t="s">
         <v>45</v>
-      </c>
-      <c r="K5" s="12" t="s">
-        <v>47</v>
       </c>
       <c r="L5" s="12" t="s">
         <v>30</v>
@@ -925,7 +922,7 @@
     <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="26" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="9" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.7109375" customWidth="1"/>
     <col min="10" max="10" width="13.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1033,22 +1030,22 @@
         <v>19</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>30</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>17</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="I4" s="9" t="s">
         <v>16</v>
@@ -1057,13 +1054,19 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
+      <c r="I5" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>23</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated 40+ and 60+ groups and schedule
</commit_message>
<xml_diff>
--- a/Savets 2026/admin/Groups.xlsx
+++ b/Savets 2026/admin/Groups.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0EA9C29-9FC4-4D49-8AE5-11666D6838D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69C1F5BB-AC13-4D2D-BE20-5A03BE465709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9120" yWindow="2190" windowWidth="15300" windowHeight="7785" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Men's 40+" sheetId="4" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="47">
   <si>
     <t>Group 1 Names</t>
   </si>
@@ -803,18 +803,18 @@
         <v>30</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>32</v>
+      <c r="A4" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>43</v>
       </c>
       <c r="C4" s="9" t="s">
         <v>36</v>
@@ -840,11 +840,11 @@
       <c r="J4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="K4" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="L4" s="5" t="s">
-        <v>23</v>
+      <c r="K4" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="L4" s="12" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -854,18 +854,6 @@
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
-      <c r="I5" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="K5" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="L5" s="12" t="s">
-        <v>30</v>
-      </c>
     </row>
     <row r="6" spans="1:12" ht="21" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C6" s="10"/>
@@ -1076,7 +1064,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -1085,45 +1073,93 @@
     <col min="4" max="4" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" s="1" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="6" t="s">
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B3" s="8" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="9" t="s">
+      <c r="C3" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="D3" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>19</v>
-      </c>
+    <row r="5" spans="1:4" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="9"/>
+      <c r="B5" s="5"/>
+    </row>
+    <row r="7" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="9"/>
+      <c r="B7" s="5"/>
+    </row>
+    <row r="8" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="6"/>
+      <c r="B8" s="8"/>
+    </row>
+    <row r="9" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="9"/>
+      <c r="B9" s="5"/>
+    </row>
+    <row r="11" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="7"/>
+    </row>
+    <row r="13" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="10"/>
+    </row>
+    <row r="14" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C14" s="10"/>
+    </row>
+    <row r="15" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="10"/>
+    </row>
+    <row r="16" spans="1:4" ht="21" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>